<commit_message>
Prima versione. Da verificare
</commit_message>
<xml_diff>
--- a/dati test.xlsx
+++ b/dati test.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eneait-my.sharepoint.com/personal/antonio_ricca_enea_it/Documents/01 - Attività/07 - POR/01 - RT/RT 4.2.1.3/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anton\PycharmProjects\HRS_manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="11_F25DC773A252ABDACC10485B591B48F45ADE58EE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D513F5F-DAB7-4862-BBDD-4CB6447292C6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E48E207A-BE60-4D61-BD7D-2D8EC1F59170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4035" yWindow="1950" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -378,1346 +378,1346 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
-        <v>0</v>
+        <v>0.29166666666666669</v>
       </c>
       <c r="B2">
-        <v>2.33</v>
+        <v>5.25</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>133.80000000000001</v>
       </c>
       <c r="D2">
-        <v>13.5</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>1.0416666666666666E-2</v>
+        <v>0.30208333333333331</v>
       </c>
       <c r="B3">
-        <v>3.1</v>
+        <v>5.63</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>174</v>
       </c>
       <c r="D3">
-        <v>13.2</v>
+        <v>14.6</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <v>2.0833333333333332E-2</v>
+        <v>0.3125</v>
       </c>
       <c r="B4">
-        <v>2.84</v>
+        <v>6.5</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>225.9</v>
       </c>
       <c r="D4">
-        <v>13.1</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>3.125E-2</v>
+        <v>0.32291666666666669</v>
       </c>
       <c r="B5">
-        <v>2.31</v>
+        <v>6.21</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>261.2</v>
       </c>
       <c r="D5">
-        <v>13.1</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>4.1666666666666664E-2</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="B6">
-        <v>2.52</v>
+        <v>8.08</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>305.3</v>
       </c>
       <c r="D6">
-        <v>12.6</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>5.2083333333333336E-2</v>
+        <v>0.34375</v>
       </c>
       <c r="B7">
-        <v>3.34</v>
+        <v>8.1199999999999992</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>353.3</v>
       </c>
       <c r="D7">
-        <v>12.5</v>
+        <v>16.100000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>6.25E-2</v>
+        <v>0.35416666666666669</v>
       </c>
       <c r="B8">
-        <v>2.31</v>
+        <v>8.5399999999999991</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>389.2</v>
       </c>
       <c r="D8">
-        <v>12.6</v>
+        <v>16.5</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>7.2916666666666671E-2</v>
+        <v>0.36458333333333331</v>
       </c>
       <c r="B9">
-        <v>2.57</v>
+        <v>8.25</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>412.4</v>
       </c>
       <c r="D9">
-        <v>12.4</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>8.3333333333333329E-2</v>
+        <v>0.375</v>
       </c>
       <c r="B10">
-        <v>3.2</v>
+        <v>8.65</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>449.7</v>
       </c>
       <c r="D10">
-        <v>12.1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>9.375E-2</v>
+        <v>0.38541666666666669</v>
       </c>
       <c r="B11">
-        <v>2.41</v>
+        <v>9</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>487.7</v>
       </c>
       <c r="D11">
-        <v>12.2</v>
+        <v>17.3</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>0.10416666666666667</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="B12">
-        <v>2.48</v>
+        <v>8.6999999999999993</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>516.20000000000005</v>
       </c>
       <c r="D12">
-        <v>12</v>
+        <v>17.600000000000001</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>0.11458333333333333</v>
+        <v>0.40625</v>
       </c>
       <c r="B13">
-        <v>2.7</v>
+        <v>8.9</v>
       </c>
       <c r="C13">
-        <v>0</v>
+        <v>545.9</v>
       </c>
       <c r="D13">
-        <v>11.9</v>
+        <v>18.100000000000001</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>0.125</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="B14">
-        <v>3.28</v>
+        <v>8.14</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>580.79999999999995</v>
       </c>
       <c r="D14">
-        <v>12</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>0.13541666666666666</v>
+        <v>0.42708333333333331</v>
       </c>
       <c r="B15">
-        <v>2.5</v>
+        <v>7.57</v>
       </c>
       <c r="C15">
-        <v>0</v>
+        <v>591.9</v>
       </c>
       <c r="D15">
-        <v>11.7</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>0.14583333333333334</v>
+        <v>0.4375</v>
       </c>
       <c r="B16">
-        <v>2.57</v>
+        <v>8.1300000000000008</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>643.1</v>
       </c>
       <c r="D16">
-        <v>11.8</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>0.15625</v>
+        <v>0.44791666666666669</v>
       </c>
       <c r="B17">
-        <v>2.57</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="C17">
-        <v>0</v>
+        <v>632.1</v>
       </c>
       <c r="D17">
-        <v>12</v>
+        <v>19.3</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>0.16666666666666666</v>
+        <v>0.45833333333333331</v>
       </c>
       <c r="B18">
-        <v>3.54</v>
+        <v>9</v>
       </c>
       <c r="C18">
-        <v>0</v>
+        <v>676.7</v>
       </c>
       <c r="D18">
-        <v>12</v>
+        <v>19.7</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>0.17708333333333334</v>
+        <v>0.46875</v>
       </c>
       <c r="B19">
-        <v>3.54</v>
+        <v>9</v>
       </c>
       <c r="C19">
-        <v>0</v>
+        <v>690.6</v>
       </c>
       <c r="D19">
-        <v>12.3</v>
+        <v>19.899999999999999</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>0.1875</v>
+        <v>0.47916666666666669</v>
       </c>
       <c r="B20">
-        <v>3.1</v>
+        <v>9</v>
       </c>
       <c r="C20">
-        <v>0</v>
+        <v>679</v>
       </c>
       <c r="D20">
-        <v>12.2</v>
+        <v>19.899999999999999</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>0.19791666666666666</v>
+        <v>0.48958333333333331</v>
       </c>
       <c r="B21">
-        <v>2.87</v>
+        <v>8.65</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>716.6</v>
       </c>
       <c r="D21">
-        <v>12.3</v>
+        <v>20.3</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
-        <v>0.20833333333333334</v>
+        <v>0.5</v>
       </c>
       <c r="B22">
-        <v>3</v>
+        <v>8.59</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>715.2</v>
       </c>
       <c r="D22">
-        <v>12.9</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>0.21875</v>
+        <v>0.51041666666666663</v>
       </c>
       <c r="B23">
-        <v>3.28</v>
+        <v>9</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>708.2</v>
       </c>
       <c r="D23">
-        <v>12.8</v>
+        <v>20.7</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
-        <v>0.22916666666666666</v>
+        <v>0.52083333333333337</v>
       </c>
       <c r="B24">
-        <v>2.39</v>
+        <v>8.0399999999999991</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>710.1</v>
       </c>
       <c r="D24">
-        <v>13</v>
+        <v>21.1</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
-        <v>0.23958333333333334</v>
+        <v>0.53125</v>
       </c>
       <c r="B25">
-        <v>3.16</v>
+        <v>8.49</v>
       </c>
       <c r="C25">
-        <v>0</v>
+        <v>728.9</v>
       </c>
       <c r="D25">
-        <v>13</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
-        <v>0.25</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="B26">
-        <v>2.31</v>
+        <v>9</v>
       </c>
       <c r="C26">
-        <v>0</v>
+        <v>709.8</v>
       </c>
       <c r="D26">
-        <v>13.4</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
-        <v>0.26041666666666669</v>
+        <v>0.55208333333333337</v>
       </c>
       <c r="B27">
-        <v>3.14</v>
+        <v>8.61</v>
       </c>
       <c r="C27">
-        <v>0</v>
+        <v>712.9</v>
       </c>
       <c r="D27">
-        <v>13.7</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>0.27083333333333331</v>
+        <v>0.5625</v>
       </c>
       <c r="B28">
-        <v>4.3499999999999996</v>
+        <v>8.57</v>
       </c>
       <c r="C28">
-        <v>44.2</v>
+        <v>696</v>
       </c>
       <c r="D28">
-        <v>13.9</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>0.28125</v>
+        <v>0.57291666666666663</v>
       </c>
       <c r="B29">
-        <v>4.1399999999999997</v>
+        <v>8.66</v>
       </c>
       <c r="C29">
-        <v>90.6</v>
+        <v>682.1</v>
       </c>
       <c r="D29">
-        <v>14.2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>0.29166666666666669</v>
+        <v>0.58333333333333337</v>
       </c>
       <c r="B30">
-        <v>5.25</v>
+        <v>8.5399999999999991</v>
       </c>
       <c r="C30">
-        <v>133.80000000000001</v>
+        <v>663.7</v>
       </c>
       <c r="D30">
-        <v>14.5</v>
+        <v>21.8</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
-        <v>0.30208333333333331</v>
+        <v>0.59375</v>
       </c>
       <c r="B31">
-        <v>5.63</v>
+        <v>9</v>
       </c>
       <c r="C31">
-        <v>174</v>
+        <v>642.20000000000005</v>
       </c>
       <c r="D31">
-        <v>14.6</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <v>0.3125</v>
+        <v>0.60416666666666663</v>
       </c>
       <c r="B32">
-        <v>6.5</v>
+        <v>9</v>
       </c>
       <c r="C32">
-        <v>225.9</v>
+        <v>628.1</v>
       </c>
       <c r="D32">
-        <v>15.2</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>0.32291666666666669</v>
+        <v>0.61458333333333337</v>
       </c>
       <c r="B33">
-        <v>6.21</v>
+        <v>9</v>
       </c>
       <c r="C33">
-        <v>261.2</v>
+        <v>602.20000000000005</v>
       </c>
       <c r="D33">
-        <v>15.2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <v>0.33333333333333331</v>
+        <v>0.625</v>
       </c>
       <c r="B34">
-        <v>8.08</v>
+        <v>8.66</v>
       </c>
       <c r="C34">
-        <v>305.3</v>
+        <v>587</v>
       </c>
       <c r="D34">
-        <v>15.5</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
-        <v>0.34375</v>
+        <v>0.63541666666666663</v>
       </c>
       <c r="B35">
-        <v>8.1199999999999992</v>
+        <v>8.92</v>
       </c>
       <c r="C35">
-        <v>353.3</v>
+        <v>563.9</v>
       </c>
       <c r="D35">
-        <v>16.100000000000001</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>0.35416666666666669</v>
+        <v>0.64583333333333337</v>
       </c>
       <c r="B36">
-        <v>8.5399999999999991</v>
+        <v>8.42</v>
       </c>
       <c r="C36">
-        <v>389.2</v>
+        <v>530.29999999999995</v>
       </c>
       <c r="D36">
-        <v>16.5</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>0.36458333333333331</v>
+        <v>0.65625</v>
       </c>
       <c r="B37">
-        <v>8.25</v>
+        <v>7.71</v>
       </c>
       <c r="C37">
-        <v>412.4</v>
+        <v>497.9</v>
       </c>
       <c r="D37">
-        <v>16.7</v>
+        <v>22</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
-        <v>0.375</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="B38">
-        <v>8.65</v>
+        <v>8.92</v>
       </c>
       <c r="C38">
-        <v>449.7</v>
+        <v>449.5</v>
       </c>
       <c r="D38">
-        <v>17</v>
+        <v>21.8</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
-        <v>0.38541666666666669</v>
+        <v>0.67708333333333337</v>
       </c>
       <c r="B39">
         <v>9</v>
       </c>
       <c r="C39">
-        <v>487.7</v>
+        <v>427.6</v>
       </c>
       <c r="D39">
-        <v>17.3</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
-        <v>0.39583333333333331</v>
+        <v>0.6875</v>
       </c>
       <c r="B40">
-        <v>8.6999999999999993</v>
+        <v>9</v>
       </c>
       <c r="C40">
-        <v>516.20000000000005</v>
+        <v>391.5</v>
       </c>
       <c r="D40">
-        <v>17.600000000000001</v>
+        <v>21.5</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
-        <v>0.40625</v>
+        <v>0.69791666666666663</v>
       </c>
       <c r="B41">
         <v>8.9</v>
       </c>
       <c r="C41">
-        <v>545.9</v>
+        <v>340.4</v>
       </c>
       <c r="D41">
-        <v>18.100000000000001</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
-        <v>0.41666666666666669</v>
+        <v>0.70833333333333337</v>
       </c>
       <c r="B42">
-        <v>8.14</v>
+        <v>8.25</v>
       </c>
       <c r="C42">
-        <v>580.79999999999995</v>
+        <v>303.89999999999998</v>
       </c>
       <c r="D42">
-        <v>18.3</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
-        <v>0.42708333333333331</v>
+        <v>0.71875</v>
       </c>
       <c r="B43">
-        <v>7.57</v>
+        <v>8.42</v>
       </c>
       <c r="C43">
-        <v>591.9</v>
+        <v>257.2</v>
       </c>
       <c r="D43">
-        <v>18.5</v>
+        <v>21.2</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
-        <v>0.4375</v>
+        <v>0.72916666666666663</v>
       </c>
       <c r="B44">
-        <v>8.1300000000000008</v>
+        <v>8.3699999999999992</v>
       </c>
       <c r="C44">
-        <v>643.1</v>
+        <v>221.5</v>
       </c>
       <c r="D44">
-        <v>18.8</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
-        <v>0.44791666666666669</v>
+        <v>0.73958333333333337</v>
       </c>
       <c r="B45">
-        <v>8.8000000000000007</v>
+        <v>8.0399999999999991</v>
       </c>
       <c r="C45">
-        <v>632.1</v>
+        <v>174.8</v>
       </c>
       <c r="D45">
-        <v>19.3</v>
+        <v>20.7</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>0.45833333333333331</v>
+        <v>0.75</v>
       </c>
       <c r="B46">
-        <v>9</v>
+        <v>8.31</v>
       </c>
       <c r="C46">
-        <v>676.7</v>
+        <v>133.1</v>
       </c>
       <c r="D46">
-        <v>19.7</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>0.46875</v>
+        <v>0.76041666666666663</v>
       </c>
       <c r="B47">
-        <v>9</v>
+        <v>7.17</v>
       </c>
       <c r="C47">
-        <v>690.6</v>
+        <v>89.9</v>
       </c>
       <c r="D47">
-        <v>19.899999999999999</v>
+        <v>20.399999999999999</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <v>0.47916666666666669</v>
+        <v>0.77083333333333337</v>
       </c>
       <c r="B48">
-        <v>9</v>
+        <v>6.48</v>
       </c>
       <c r="C48">
-        <v>679</v>
+        <v>45.4</v>
       </c>
       <c r="D48">
-        <v>19.899999999999999</v>
+        <v>20.100000000000001</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
-        <v>0.48958333333333331</v>
+        <v>0.78125</v>
       </c>
       <c r="B49">
-        <v>8.65</v>
+        <v>7.34</v>
       </c>
       <c r="C49">
-        <v>716.6</v>
+        <v>0</v>
       </c>
       <c r="D49">
-        <v>20.3</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>0.5</v>
+        <v>0.79166666666666663</v>
       </c>
       <c r="B50">
-        <v>8.59</v>
+        <v>6.5</v>
       </c>
       <c r="C50">
-        <v>715.2</v>
+        <v>0</v>
       </c>
       <c r="D50">
-        <v>20.5</v>
+        <v>19.5</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>0.51041666666666663</v>
+        <v>0.80208333333333337</v>
       </c>
       <c r="B51">
-        <v>9</v>
+        <v>6.29</v>
       </c>
       <c r="C51">
-        <v>708.2</v>
+        <v>0</v>
       </c>
       <c r="D51">
-        <v>20.7</v>
+        <v>19</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <v>0.52083333333333337</v>
+        <v>0.8125</v>
       </c>
       <c r="B52">
-        <v>8.0399999999999991</v>
+        <v>5.72</v>
       </c>
       <c r="C52">
-        <v>710.1</v>
+        <v>0</v>
       </c>
       <c r="D52">
-        <v>21.1</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>0.53125</v>
+        <v>0.82291666666666663</v>
       </c>
       <c r="B53">
-        <v>8.49</v>
+        <v>5.13</v>
       </c>
       <c r="C53">
-        <v>728.9</v>
+        <v>0</v>
       </c>
       <c r="D53">
-        <v>21.4</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <v>0.54166666666666663</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="B54">
-        <v>9</v>
+        <v>5.87</v>
       </c>
       <c r="C54">
-        <v>709.8</v>
+        <v>0</v>
       </c>
       <c r="D54">
-        <v>21.4</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <v>0.55208333333333337</v>
+        <v>0.84375</v>
       </c>
       <c r="B55">
-        <v>8.61</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="C55">
-        <v>712.9</v>
+        <v>0</v>
       </c>
       <c r="D55">
-        <v>21.4</v>
+        <v>17.899999999999999</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>0.5625</v>
+        <v>0.85416666666666663</v>
       </c>
       <c r="B56">
-        <v>8.57</v>
+        <v>5.4</v>
       </c>
       <c r="C56">
-        <v>696</v>
+        <v>0</v>
       </c>
       <c r="D56">
-        <v>21.6</v>
+        <v>17.600000000000001</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
-        <v>0.57291666666666663</v>
+        <v>0.86458333333333337</v>
       </c>
       <c r="B57">
-        <v>8.66</v>
+        <v>4.78</v>
       </c>
       <c r="C57">
-        <v>682.1</v>
+        <v>0</v>
       </c>
       <c r="D57">
-        <v>22</v>
+        <v>17.3</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
-        <v>0.58333333333333337</v>
+        <v>0.875</v>
       </c>
       <c r="B58">
-        <v>8.5399999999999991</v>
+        <v>4.0599999999999996</v>
       </c>
       <c r="C58">
-        <v>663.7</v>
+        <v>0</v>
       </c>
       <c r="D58">
-        <v>21.8</v>
+        <v>17.100000000000001</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
-        <v>0.59375</v>
+        <v>0.88541666666666663</v>
       </c>
       <c r="B59">
-        <v>9</v>
+        <v>3.47</v>
       </c>
       <c r="C59">
-        <v>642.20000000000005</v>
+        <v>0</v>
       </c>
       <c r="D59">
-        <v>21.9</v>
+        <v>16.600000000000001</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>0.60416666666666663</v>
+        <v>0.89583333333333337</v>
       </c>
       <c r="B60">
-        <v>9</v>
+        <v>3.29</v>
       </c>
       <c r="C60">
-        <v>628.1</v>
+        <v>0</v>
       </c>
       <c r="D60">
-        <v>21.9</v>
+        <v>16.3</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <v>0.61458333333333337</v>
+        <v>0.90625</v>
       </c>
       <c r="B61">
-        <v>9</v>
+        <v>2.8</v>
       </c>
       <c r="C61">
-        <v>602.20000000000005</v>
+        <v>0</v>
       </c>
       <c r="D61">
-        <v>22</v>
+        <v>16</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
-        <v>0.625</v>
+        <v>0.91666666666666663</v>
       </c>
       <c r="B62">
-        <v>8.66</v>
+        <v>3.5</v>
       </c>
       <c r="C62">
-        <v>587</v>
+        <v>0</v>
       </c>
       <c r="D62">
-        <v>21.9</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
-        <v>0.63541666666666663</v>
+        <v>0.92708333333333337</v>
       </c>
       <c r="B63">
-        <v>8.92</v>
+        <v>2.79</v>
       </c>
       <c r="C63">
-        <v>563.9</v>
+        <v>0</v>
       </c>
       <c r="D63">
-        <v>21.9</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
-        <v>0.64583333333333337</v>
+        <v>0.9375</v>
       </c>
       <c r="B64">
-        <v>8.42</v>
+        <v>3.15</v>
       </c>
       <c r="C64">
-        <v>530.29999999999995</v>
+        <v>0</v>
       </c>
       <c r="D64">
-        <v>22.1</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <v>0.65625</v>
+        <v>0.94791666666666663</v>
       </c>
       <c r="B65">
-        <v>7.71</v>
+        <v>2.31</v>
       </c>
       <c r="C65">
-        <v>497.9</v>
+        <v>0</v>
       </c>
       <c r="D65">
-        <v>22</v>
+        <v>14.6</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <v>0.66666666666666663</v>
+        <v>0.95833333333333337</v>
       </c>
       <c r="B66">
-        <v>8.92</v>
+        <v>2.8</v>
       </c>
       <c r="C66">
-        <v>449.5</v>
+        <v>0</v>
       </c>
       <c r="D66">
-        <v>21.8</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
-        <v>0.67708333333333337</v>
+        <v>0.96875</v>
       </c>
       <c r="B67">
-        <v>9</v>
+        <v>3.16</v>
       </c>
       <c r="C67">
-        <v>427.6</v>
+        <v>0</v>
       </c>
       <c r="D67">
-        <v>21.9</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <v>0.6875</v>
+        <v>0.97916666666666663</v>
       </c>
       <c r="B68">
-        <v>9</v>
+        <v>2.61</v>
       </c>
       <c r="C68">
-        <v>391.5</v>
+        <v>0</v>
       </c>
       <c r="D68">
-        <v>21.5</v>
+        <v>13.8</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <v>0.69791666666666663</v>
+        <v>0.98958333333333337</v>
       </c>
       <c r="B69">
-        <v>8.9</v>
+        <v>3.11</v>
       </c>
       <c r="C69">
-        <v>340.4</v>
+        <v>0</v>
       </c>
       <c r="D69">
-        <v>21.4</v>
+        <v>13.9</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <v>0.70833333333333337</v>
+        <v>0</v>
       </c>
       <c r="B70">
-        <v>8.25</v>
+        <v>2.33</v>
       </c>
       <c r="C70">
-        <v>303.89999999999998</v>
+        <v>0</v>
       </c>
       <c r="D70">
-        <v>21.4</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <v>0.71875</v>
+        <v>1.0416666666666666E-2</v>
       </c>
       <c r="B71">
-        <v>8.42</v>
+        <v>3.1</v>
       </c>
       <c r="C71">
-        <v>257.2</v>
+        <v>0</v>
       </c>
       <c r="D71">
-        <v>21.2</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
-        <v>0.72916666666666663</v>
+        <v>2.0833333333333332E-2</v>
       </c>
       <c r="B72">
-        <v>8.3699999999999992</v>
+        <v>2.84</v>
       </c>
       <c r="C72">
-        <v>221.5</v>
+        <v>0</v>
       </c>
       <c r="D72">
-        <v>20.8</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
-        <v>0.73958333333333337</v>
+        <v>3.125E-2</v>
       </c>
       <c r="B73">
-        <v>8.0399999999999991</v>
+        <v>2.31</v>
       </c>
       <c r="C73">
-        <v>174.8</v>
+        <v>0</v>
       </c>
       <c r="D73">
-        <v>20.7</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
-        <v>0.75</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="B74">
-        <v>8.31</v>
+        <v>2.52</v>
       </c>
       <c r="C74">
-        <v>133.1</v>
+        <v>0</v>
       </c>
       <c r="D74">
-        <v>20.5</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
-        <v>0.76041666666666663</v>
+        <v>5.2083333333333336E-2</v>
       </c>
       <c r="B75">
-        <v>7.17</v>
+        <v>3.34</v>
       </c>
       <c r="C75">
-        <v>89.9</v>
+        <v>0</v>
       </c>
       <c r="D75">
-        <v>20.399999999999999</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
-        <v>0.77083333333333337</v>
+        <v>6.25E-2</v>
       </c>
       <c r="B76">
-        <v>6.48</v>
+        <v>2.31</v>
       </c>
       <c r="C76">
-        <v>45.4</v>
+        <v>0</v>
       </c>
       <c r="D76">
-        <v>20.100000000000001</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
-        <v>0.78125</v>
+        <v>7.2916666666666671E-2</v>
       </c>
       <c r="B77">
-        <v>7.34</v>
+        <v>2.57</v>
       </c>
       <c r="C77">
         <v>0</v>
       </c>
       <c r="D77">
-        <v>19.8</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
-        <v>0.79166666666666663</v>
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="B78">
-        <v>6.5</v>
+        <v>3.2</v>
       </c>
       <c r="C78">
         <v>0</v>
       </c>
       <c r="D78">
-        <v>19.5</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
-        <v>0.80208333333333337</v>
+        <v>9.375E-2</v>
       </c>
       <c r="B79">
-        <v>6.29</v>
+        <v>2.41</v>
       </c>
       <c r="C79">
         <v>0</v>
       </c>
       <c r="D79">
-        <v>19</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
-        <v>0.8125</v>
+        <v>0.10416666666666667</v>
       </c>
       <c r="B80">
-        <v>5.72</v>
+        <v>2.48</v>
       </c>
       <c r="C80">
         <v>0</v>
       </c>
       <c r="D80">
-        <v>18.8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
-        <v>0.82291666666666663</v>
+        <v>0.11458333333333333</v>
       </c>
       <c r="B81">
-        <v>5.13</v>
+        <v>2.7</v>
       </c>
       <c r="C81">
         <v>0</v>
       </c>
       <c r="D81">
-        <v>18.5</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
-        <v>0.83333333333333337</v>
+        <v>0.125</v>
       </c>
       <c r="B82">
-        <v>5.87</v>
+        <v>3.28</v>
       </c>
       <c r="C82">
         <v>0</v>
       </c>
       <c r="D82">
-        <v>18.3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
-        <v>0.84375</v>
+        <v>0.13541666666666666</v>
       </c>
       <c r="B83">
-        <v>4.8499999999999996</v>
+        <v>2.5</v>
       </c>
       <c r="C83">
         <v>0</v>
       </c>
       <c r="D83">
-        <v>17.899999999999999</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
-        <v>0.85416666666666663</v>
+        <v>0.14583333333333334</v>
       </c>
       <c r="B84">
-        <v>5.4</v>
+        <v>2.57</v>
       </c>
       <c r="C84">
         <v>0</v>
       </c>
       <c r="D84">
-        <v>17.600000000000001</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
-        <v>0.86458333333333337</v>
+        <v>0.15625</v>
       </c>
       <c r="B85">
-        <v>4.78</v>
+        <v>2.57</v>
       </c>
       <c r="C85">
         <v>0</v>
       </c>
       <c r="D85">
-        <v>17.3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
-        <v>0.875</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="B86">
-        <v>4.0599999999999996</v>
+        <v>3.54</v>
       </c>
       <c r="C86">
         <v>0</v>
       </c>
       <c r="D86">
-        <v>17.100000000000001</v>
+        <v>12</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
-        <v>0.88541666666666663</v>
+        <v>0.17708333333333334</v>
       </c>
       <c r="B87">
-        <v>3.47</v>
+        <v>3.54</v>
       </c>
       <c r="C87">
         <v>0</v>
       </c>
       <c r="D87">
-        <v>16.600000000000001</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
-        <v>0.89583333333333337</v>
+        <v>0.1875</v>
       </c>
       <c r="B88">
-        <v>3.29</v>
+        <v>3.1</v>
       </c>
       <c r="C88">
         <v>0</v>
       </c>
       <c r="D88">
-        <v>16.3</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
-        <v>0.90625</v>
+        <v>0.19791666666666666</v>
       </c>
       <c r="B89">
-        <v>2.8</v>
+        <v>2.87</v>
       </c>
       <c r="C89">
         <v>0</v>
       </c>
       <c r="D89">
-        <v>16</v>
+        <v>12.3</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
-        <v>0.91666666666666663</v>
+        <v>0.20833333333333334</v>
       </c>
       <c r="B90">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="C90">
         <v>0</v>
       </c>
       <c r="D90">
-        <v>15.8</v>
+        <v>12.9</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
-        <v>0.92708333333333337</v>
+        <v>0.21875</v>
       </c>
       <c r="B91">
-        <v>2.79</v>
+        <v>3.28</v>
       </c>
       <c r="C91">
         <v>0</v>
       </c>
       <c r="D91">
-        <v>15.4</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
-        <v>0.9375</v>
+        <v>0.22916666666666666</v>
       </c>
       <c r="B92">
-        <v>3.15</v>
+        <v>2.39</v>
       </c>
       <c r="C92">
         <v>0</v>
       </c>
       <c r="D92">
-        <v>15.2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
-        <v>0.94791666666666663</v>
+        <v>0.23958333333333334</v>
       </c>
       <c r="B93">
-        <v>2.31</v>
+        <v>3.16</v>
       </c>
       <c r="C93">
         <v>0</v>
       </c>
       <c r="D93">
-        <v>14.6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
-        <v>0.95833333333333337</v>
+        <v>0.25</v>
       </c>
       <c r="B94">
-        <v>2.8</v>
+        <v>2.31</v>
       </c>
       <c r="C94">
         <v>0</v>
       </c>
       <c r="D94">
-        <v>14.4</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
-        <v>0.96875</v>
+        <v>0.26041666666666669</v>
       </c>
       <c r="B95">
-        <v>3.16</v>
+        <v>3.14</v>
       </c>
       <c r="C95">
         <v>0</v>
       </c>
       <c r="D95">
-        <v>14.3</v>
+        <v>13.7</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
-        <v>0.97916666666666663</v>
+        <v>0.27083333333333331</v>
       </c>
       <c r="B96">
-        <v>2.61</v>
+        <v>4.3499999999999996</v>
       </c>
       <c r="C96">
-        <v>0</v>
+        <v>44.2</v>
       </c>
       <c r="D96">
-        <v>13.8</v>
+        <v>13.9</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
-        <v>0.98958333333333337</v>
+        <v>0.28125</v>
       </c>
       <c r="B97">
-        <v>3.11</v>
+        <v>4.1399999999999997</v>
       </c>
       <c r="C97">
-        <v>0</v>
+        <v>90.6</v>
       </c>
       <c r="D97">
-        <v>13.9</v>
+        <v>14.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gestione delle ricariche multiple, aggiunta possibilità di orizzonte temporale maggiore di 1 giorno
</commit_message>
<xml_diff>
--- a/dati test.xlsx
+++ b/dati test.xlsx
@@ -8,17 +8,28 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anton\PycharmProjects\HRS_manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E48E207A-BE60-4D61-BD7D-2D8EC1F59170}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93852D5-C1D5-4D3D-9732-61D1F370D3EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -381,7 +392,7 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="B2">
-        <v>5.25</v>
+        <v>1.44</v>
       </c>
       <c r="C2">
         <v>133.80000000000001</v>
@@ -395,7 +406,7 @@
         <v>0.30208333333333331</v>
       </c>
       <c r="B3">
-        <v>5.63</v>
+        <v>1.5</v>
       </c>
       <c r="C3">
         <v>174</v>
@@ -409,7 +420,7 @@
         <v>0.3125</v>
       </c>
       <c r="B4">
-        <v>6.5</v>
+        <v>1.59</v>
       </c>
       <c r="C4">
         <v>225.9</v>
@@ -423,7 +434,7 @@
         <v>0.32291666666666669</v>
       </c>
       <c r="B5">
-        <v>6.21</v>
+        <v>1.47</v>
       </c>
       <c r="C5">
         <v>261.2</v>
@@ -437,7 +448,7 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="B6">
-        <v>8.08</v>
+        <v>1.55</v>
       </c>
       <c r="C6">
         <v>305.3</v>
@@ -451,7 +462,7 @@
         <v>0.34375</v>
       </c>
       <c r="B7">
-        <v>8.1199999999999992</v>
+        <v>1.36</v>
       </c>
       <c r="C7">
         <v>353.3</v>
@@ -465,7 +476,7 @@
         <v>0.35416666666666669</v>
       </c>
       <c r="B8">
-        <v>8.5399999999999991</v>
+        <v>1.42</v>
       </c>
       <c r="C8">
         <v>389.2</v>
@@ -479,7 +490,7 @@
         <v>0.36458333333333331</v>
       </c>
       <c r="B9">
-        <v>8.25</v>
+        <v>1.48</v>
       </c>
       <c r="C9">
         <v>412.4</v>
@@ -493,7 +504,7 @@
         <v>0.375</v>
       </c>
       <c r="B10">
-        <v>8.65</v>
+        <v>1.42</v>
       </c>
       <c r="C10">
         <v>449.7</v>
@@ -507,7 +518,7 @@
         <v>0.38541666666666669</v>
       </c>
       <c r="B11">
-        <v>9</v>
+        <v>1.32</v>
       </c>
       <c r="C11">
         <v>487.7</v>
@@ -521,7 +532,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="B12">
-        <v>8.6999999999999993</v>
+        <v>1.56</v>
       </c>
       <c r="C12">
         <v>516.20000000000005</v>
@@ -535,7 +546,7 @@
         <v>0.40625</v>
       </c>
       <c r="B13">
-        <v>8.9</v>
+        <v>1.21</v>
       </c>
       <c r="C13">
         <v>545.9</v>
@@ -549,7 +560,7 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="B14">
-        <v>8.14</v>
+        <v>1.45</v>
       </c>
       <c r="C14">
         <v>580.79999999999995</v>
@@ -563,7 +574,7 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="B15">
-        <v>7.57</v>
+        <v>2</v>
       </c>
       <c r="C15">
         <v>591.9</v>
@@ -577,7 +588,7 @@
         <v>0.4375</v>
       </c>
       <c r="B16">
-        <v>8.1300000000000008</v>
+        <v>2.06</v>
       </c>
       <c r="C16">
         <v>643.1</v>
@@ -591,7 +602,7 @@
         <v>0.44791666666666669</v>
       </c>
       <c r="B17">
-        <v>8.8000000000000007</v>
+        <v>1.41</v>
       </c>
       <c r="C17">
         <v>632.1</v>
@@ -605,7 +616,7 @@
         <v>0.45833333333333331</v>
       </c>
       <c r="B18">
-        <v>9</v>
+        <v>1.42</v>
       </c>
       <c r="C18">
         <v>676.7</v>
@@ -619,7 +630,7 @@
         <v>0.46875</v>
       </c>
       <c r="B19">
-        <v>9</v>
+        <v>1.24</v>
       </c>
       <c r="C19">
         <v>690.6</v>
@@ -633,7 +644,7 @@
         <v>0.47916666666666669</v>
       </c>
       <c r="B20">
-        <v>9</v>
+        <v>1.5</v>
       </c>
       <c r="C20">
         <v>679</v>
@@ -647,7 +658,7 @@
         <v>0.48958333333333331</v>
       </c>
       <c r="B21">
-        <v>8.65</v>
+        <v>1.36</v>
       </c>
       <c r="C21">
         <v>716.6</v>
@@ -661,7 +672,7 @@
         <v>0.5</v>
       </c>
       <c r="B22">
-        <v>8.59</v>
+        <v>1.55</v>
       </c>
       <c r="C22">
         <v>715.2</v>
@@ -675,7 +686,7 @@
         <v>0.51041666666666663</v>
       </c>
       <c r="B23">
-        <v>9</v>
+        <v>1.58</v>
       </c>
       <c r="C23">
         <v>708.2</v>
@@ -689,7 +700,7 @@
         <v>0.52083333333333337</v>
       </c>
       <c r="B24">
-        <v>8.0399999999999991</v>
+        <v>2</v>
       </c>
       <c r="C24">
         <v>710.1</v>
@@ -703,7 +714,7 @@
         <v>0.53125</v>
       </c>
       <c r="B25">
-        <v>8.49</v>
+        <v>1.41</v>
       </c>
       <c r="C25">
         <v>728.9</v>
@@ -717,7 +728,7 @@
         <v>0.54166666666666663</v>
       </c>
       <c r="B26">
-        <v>9</v>
+        <v>1.46</v>
       </c>
       <c r="C26">
         <v>709.8</v>
@@ -731,7 +742,7 @@
         <v>0.55208333333333337</v>
       </c>
       <c r="B27">
-        <v>8.61</v>
+        <v>1.51</v>
       </c>
       <c r="C27">
         <v>712.9</v>
@@ -745,7 +756,7 @@
         <v>0.5625</v>
       </c>
       <c r="B28">
-        <v>8.57</v>
+        <v>1.42</v>
       </c>
       <c r="C28">
         <v>696</v>
@@ -759,7 +770,7 @@
         <v>0.57291666666666663</v>
       </c>
       <c r="B29">
-        <v>8.66</v>
+        <v>1.37</v>
       </c>
       <c r="C29">
         <v>682.1</v>
@@ -773,7 +784,7 @@
         <v>0.58333333333333337</v>
       </c>
       <c r="B30">
-        <v>8.5399999999999991</v>
+        <v>6</v>
       </c>
       <c r="C30">
         <v>663.7</v>
@@ -787,7 +798,7 @@
         <v>0.59375</v>
       </c>
       <c r="B31">
-        <v>9</v>
+        <v>6.16</v>
       </c>
       <c r="C31">
         <v>642.20000000000005</v>
@@ -801,7 +812,7 @@
         <v>0.60416666666666663</v>
       </c>
       <c r="B32">
-        <v>9</v>
+        <v>5.12</v>
       </c>
       <c r="C32">
         <v>628.1</v>
@@ -815,7 +826,7 @@
         <v>0.61458333333333337</v>
       </c>
       <c r="B33">
-        <v>9</v>
+        <v>7.07</v>
       </c>
       <c r="C33">
         <v>602.20000000000005</v>
@@ -829,7 +840,7 @@
         <v>0.625</v>
       </c>
       <c r="B34">
-        <v>8.66</v>
+        <v>7</v>
       </c>
       <c r="C34">
         <v>587</v>
@@ -843,7 +854,7 @@
         <v>0.63541666666666663</v>
       </c>
       <c r="B35">
-        <v>8.92</v>
+        <v>7.01</v>
       </c>
       <c r="C35">
         <v>563.9</v>
@@ -857,7 +868,7 @@
         <v>0.64583333333333337</v>
       </c>
       <c r="B36">
-        <v>8.42</v>
+        <v>7.34</v>
       </c>
       <c r="C36">
         <v>530.29999999999995</v>
@@ -871,7 +882,7 @@
         <v>0.65625</v>
       </c>
       <c r="B37">
-        <v>7.71</v>
+        <v>7.45</v>
       </c>
       <c r="C37">
         <v>497.9</v>
@@ -885,7 +896,7 @@
         <v>0.66666666666666663</v>
       </c>
       <c r="B38">
-        <v>8.92</v>
+        <v>9.02</v>
       </c>
       <c r="C38">
         <v>449.5</v>
@@ -899,7 +910,7 @@
         <v>0.67708333333333337</v>
       </c>
       <c r="B39">
-        <v>9</v>
+        <v>8.43</v>
       </c>
       <c r="C39">
         <v>427.6</v>
@@ -913,7 +924,7 @@
         <v>0.6875</v>
       </c>
       <c r="B40">
-        <v>9</v>
+        <v>9.33</v>
       </c>
       <c r="C40">
         <v>391.5</v>
@@ -927,7 +938,7 @@
         <v>0.69791666666666663</v>
       </c>
       <c r="B41">
-        <v>8.9</v>
+        <v>10.23</v>
       </c>
       <c r="C41">
         <v>340.4</v>
@@ -941,7 +952,7 @@
         <v>0.70833333333333337</v>
       </c>
       <c r="B42">
-        <v>8.25</v>
+        <v>9.42</v>
       </c>
       <c r="C42">
         <v>303.89999999999998</v>
@@ -955,7 +966,7 @@
         <v>0.71875</v>
       </c>
       <c r="B43">
-        <v>8.42</v>
+        <v>9.41</v>
       </c>
       <c r="C43">
         <v>257.2</v>
@@ -969,7 +980,7 @@
         <v>0.72916666666666663</v>
       </c>
       <c r="B44">
-        <v>8.3699999999999992</v>
+        <v>9.06</v>
       </c>
       <c r="C44">
         <v>221.5</v>
@@ -983,7 +994,7 @@
         <v>0.73958333333333337</v>
       </c>
       <c r="B45">
-        <v>8.0399999999999991</v>
+        <v>10.53</v>
       </c>
       <c r="C45">
         <v>174.8</v>
@@ -997,7 +1008,7 @@
         <v>0.75</v>
       </c>
       <c r="B46">
-        <v>8.31</v>
+        <v>9.33</v>
       </c>
       <c r="C46">
         <v>133.1</v>
@@ -1011,7 +1022,7 @@
         <v>0.76041666666666663</v>
       </c>
       <c r="B47">
-        <v>7.17</v>
+        <v>8.2100000000000009</v>
       </c>
       <c r="C47">
         <v>89.9</v>
@@ -1025,7 +1036,7 @@
         <v>0.77083333333333337</v>
       </c>
       <c r="B48">
-        <v>6.48</v>
+        <v>7.33</v>
       </c>
       <c r="C48">
         <v>45.4</v>
@@ -1039,7 +1050,7 @@
         <v>0.78125</v>
       </c>
       <c r="B49">
-        <v>7.34</v>
+        <v>7.28</v>
       </c>
       <c r="C49">
         <v>0</v>
@@ -1053,7 +1064,7 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="B50">
-        <v>6.5</v>
+        <v>5.52</v>
       </c>
       <c r="C50">
         <v>0</v>
@@ -1067,7 +1078,7 @@
         <v>0.80208333333333337</v>
       </c>
       <c r="B51">
-        <v>6.29</v>
+        <v>7.11</v>
       </c>
       <c r="C51">
         <v>0</v>
@@ -1081,7 +1092,7 @@
         <v>0.8125</v>
       </c>
       <c r="B52">
-        <v>5.72</v>
+        <v>6.17</v>
       </c>
       <c r="C52">
         <v>0</v>
@@ -1095,7 +1106,7 @@
         <v>0.82291666666666663</v>
       </c>
       <c r="B53">
-        <v>5.13</v>
+        <v>7.12</v>
       </c>
       <c r="C53">
         <v>0</v>
@@ -1109,7 +1120,7 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="B54">
-        <v>5.87</v>
+        <v>6.19</v>
       </c>
       <c r="C54">
         <v>0</v>
@@ -1123,7 +1134,7 @@
         <v>0.84375</v>
       </c>
       <c r="B55">
-        <v>4.8499999999999996</v>
+        <v>7.02</v>
       </c>
       <c r="C55">
         <v>0</v>
@@ -1137,7 +1148,7 @@
         <v>0.85416666666666663</v>
       </c>
       <c r="B56">
-        <v>5.4</v>
+        <v>6.4</v>
       </c>
       <c r="C56">
         <v>0</v>
@@ -1151,7 +1162,7 @@
         <v>0.86458333333333337</v>
       </c>
       <c r="B57">
-        <v>4.78</v>
+        <v>6.22</v>
       </c>
       <c r="C57">
         <v>0</v>
@@ -1165,7 +1176,7 @@
         <v>0.875</v>
       </c>
       <c r="B58">
-        <v>4.0599999999999996</v>
+        <v>9.06</v>
       </c>
       <c r="C58">
         <v>0</v>
@@ -1179,7 +1190,7 @@
         <v>0.88541666666666663</v>
       </c>
       <c r="B59">
-        <v>3.47</v>
+        <v>9.02</v>
       </c>
       <c r="C59">
         <v>0</v>
@@ -1193,7 +1204,7 @@
         <v>0.89583333333333337</v>
       </c>
       <c r="B60">
-        <v>3.29</v>
+        <v>9.3000000000000007</v>
       </c>
       <c r="C60">
         <v>0</v>
@@ -1207,7 +1218,7 @@
         <v>0.90625</v>
       </c>
       <c r="B61">
-        <v>2.8</v>
+        <v>9.35</v>
       </c>
       <c r="C61">
         <v>0</v>
@@ -1221,7 +1232,7 @@
         <v>0.91666666666666663</v>
       </c>
       <c r="B62">
-        <v>3.5</v>
+        <v>9.49</v>
       </c>
       <c r="C62">
         <v>0</v>
@@ -1235,7 +1246,7 @@
         <v>0.92708333333333337</v>
       </c>
       <c r="B63">
-        <v>2.79</v>
+        <v>9.5500000000000007</v>
       </c>
       <c r="C63">
         <v>0</v>
@@ -1249,7 +1260,7 @@
         <v>0.9375</v>
       </c>
       <c r="B64">
-        <v>3.15</v>
+        <v>9.11</v>
       </c>
       <c r="C64">
         <v>0</v>
@@ -1263,7 +1274,7 @@
         <v>0.94791666666666663</v>
       </c>
       <c r="B65">
-        <v>2.31</v>
+        <v>9.39</v>
       </c>
       <c r="C65">
         <v>0</v>
@@ -1277,7 +1288,7 @@
         <v>0.95833333333333337</v>
       </c>
       <c r="B66">
-        <v>2.8</v>
+        <v>8.35</v>
       </c>
       <c r="C66">
         <v>0</v>
@@ -1291,7 +1302,7 @@
         <v>0.96875</v>
       </c>
       <c r="B67">
-        <v>3.16</v>
+        <v>8.25</v>
       </c>
       <c r="C67">
         <v>0</v>
@@ -1305,7 +1316,7 @@
         <v>0.97916666666666663</v>
       </c>
       <c r="B68">
-        <v>2.61</v>
+        <v>8.1300000000000008</v>
       </c>
       <c r="C68">
         <v>0</v>
@@ -1319,7 +1330,7 @@
         <v>0.98958333333333337</v>
       </c>
       <c r="B69">
-        <v>3.11</v>
+        <v>8.2899999999999991</v>
       </c>
       <c r="C69">
         <v>0</v>
@@ -1333,7 +1344,7 @@
         <v>0</v>
       </c>
       <c r="B70">
-        <v>2.33</v>
+        <v>6.35</v>
       </c>
       <c r="C70">
         <v>0</v>
@@ -1347,7 +1358,7 @@
         <v>1.0416666666666666E-2</v>
       </c>
       <c r="B71">
-        <v>3.1</v>
+        <v>5.43</v>
       </c>
       <c r="C71">
         <v>0</v>
@@ -1361,7 +1372,7 @@
         <v>2.0833333333333332E-2</v>
       </c>
       <c r="B72">
-        <v>2.84</v>
+        <v>6.28</v>
       </c>
       <c r="C72">
         <v>0</v>
@@ -1375,7 +1386,7 @@
         <v>3.125E-2</v>
       </c>
       <c r="B73">
-        <v>2.31</v>
+        <v>6.44</v>
       </c>
       <c r="C73">
         <v>0</v>
@@ -1389,7 +1400,7 @@
         <v>4.1666666666666664E-2</v>
       </c>
       <c r="B74">
-        <v>2.52</v>
+        <v>6.05</v>
       </c>
       <c r="C74">
         <v>0</v>
@@ -1403,7 +1414,7 @@
         <v>5.2083333333333336E-2</v>
       </c>
       <c r="B75">
-        <v>3.34</v>
+        <v>1.55</v>
       </c>
       <c r="C75">
         <v>0</v>
@@ -1417,7 +1428,7 @@
         <v>6.25E-2</v>
       </c>
       <c r="B76">
-        <v>2.31</v>
+        <v>1.39</v>
       </c>
       <c r="C76">
         <v>0</v>
@@ -1431,7 +1442,7 @@
         <v>7.2916666666666671E-2</v>
       </c>
       <c r="B77">
-        <v>2.57</v>
+        <v>1.3</v>
       </c>
       <c r="C77">
         <v>0</v>
@@ -1445,7 +1456,7 @@
         <v>8.3333333333333329E-2</v>
       </c>
       <c r="B78">
-        <v>3.2</v>
+        <v>1.45</v>
       </c>
       <c r="C78">
         <v>0</v>
@@ -1459,7 +1470,7 @@
         <v>9.375E-2</v>
       </c>
       <c r="B79">
-        <v>2.41</v>
+        <v>1.52</v>
       </c>
       <c r="C79">
         <v>0</v>
@@ -1473,7 +1484,7 @@
         <v>0.10416666666666667</v>
       </c>
       <c r="B80">
-        <v>2.48</v>
+        <v>2.0499999999999998</v>
       </c>
       <c r="C80">
         <v>0</v>
@@ -1487,7 +1498,7 @@
         <v>0.11458333333333333</v>
       </c>
       <c r="B81">
-        <v>2.7</v>
+        <v>1.39</v>
       </c>
       <c r="C81">
         <v>0</v>
@@ -1501,7 +1512,7 @@
         <v>0.125</v>
       </c>
       <c r="B82">
-        <v>3.28</v>
+        <v>2.0499999999999998</v>
       </c>
       <c r="C82">
         <v>0</v>
@@ -1515,7 +1526,7 @@
         <v>0.13541666666666666</v>
       </c>
       <c r="B83">
-        <v>2.5</v>
+        <v>1.52</v>
       </c>
       <c r="C83">
         <v>0</v>
@@ -1529,7 +1540,7 @@
         <v>0.14583333333333334</v>
       </c>
       <c r="B84">
-        <v>2.57</v>
+        <v>1.45</v>
       </c>
       <c r="C84">
         <v>0</v>
@@ -1543,7 +1554,7 @@
         <v>0.15625</v>
       </c>
       <c r="B85">
-        <v>2.57</v>
+        <v>1.42</v>
       </c>
       <c r="C85">
         <v>0</v>
@@ -1557,7 +1568,7 @@
         <v>0.16666666666666666</v>
       </c>
       <c r="B86">
-        <v>3.54</v>
+        <v>1.52</v>
       </c>
       <c r="C86">
         <v>0</v>
@@ -1571,7 +1582,7 @@
         <v>0.17708333333333334</v>
       </c>
       <c r="B87">
-        <v>3.54</v>
+        <v>2.08</v>
       </c>
       <c r="C87">
         <v>0</v>
@@ -1585,7 +1596,7 @@
         <v>0.1875</v>
       </c>
       <c r="B88">
-        <v>3.1</v>
+        <v>1.33</v>
       </c>
       <c r="C88">
         <v>0</v>
@@ -1599,7 +1610,7 @@
         <v>0.19791666666666666</v>
       </c>
       <c r="B89">
-        <v>2.87</v>
+        <v>1.47</v>
       </c>
       <c r="C89">
         <v>0</v>
@@ -1613,7 +1624,7 @@
         <v>0.20833333333333334</v>
       </c>
       <c r="B90">
-        <v>3</v>
+        <v>1.49</v>
       </c>
       <c r="C90">
         <v>0</v>
@@ -1627,7 +1638,7 @@
         <v>0.21875</v>
       </c>
       <c r="B91">
-        <v>3.28</v>
+        <v>1.47</v>
       </c>
       <c r="C91">
         <v>0</v>
@@ -1641,7 +1652,7 @@
         <v>0.22916666666666666</v>
       </c>
       <c r="B92">
-        <v>2.39</v>
+        <v>1.51</v>
       </c>
       <c r="C92">
         <v>0</v>
@@ -1655,7 +1666,7 @@
         <v>0.23958333333333334</v>
       </c>
       <c r="B93">
-        <v>3.16</v>
+        <v>1.51</v>
       </c>
       <c r="C93">
         <v>0</v>
@@ -1669,7 +1680,7 @@
         <v>0.25</v>
       </c>
       <c r="B94">
-        <v>2.31</v>
+        <v>1.45</v>
       </c>
       <c r="C94">
         <v>0</v>
@@ -1683,7 +1694,7 @@
         <v>0.26041666666666669</v>
       </c>
       <c r="B95">
-        <v>3.14</v>
+        <v>1.58</v>
       </c>
       <c r="C95">
         <v>0</v>
@@ -1697,7 +1708,7 @@
         <v>0.27083333333333331</v>
       </c>
       <c r="B96">
-        <v>4.3499999999999996</v>
+        <v>1.42</v>
       </c>
       <c r="C96">
         <v>44.2</v>
@@ -1711,7 +1722,7 @@
         <v>0.28125</v>
       </c>
       <c r="B97">
-        <v>4.1399999999999997</v>
+        <v>1.56</v>
       </c>
       <c r="C97">
         <v>90.6</v>

</xml_diff>

<commit_message>
Ottimizzato l'esercizio, creato il generatore del profilo annuale. bisogna solo impostare lo studio
</commit_message>
<xml_diff>
--- a/dati test.xlsx
+++ b/dati test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anton\PycharmProjects\HRS_manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B93852D5-C1D5-4D3D-9732-61D1F370D3EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77F1FA06-101C-4A67-A6B0-F7685EB2FFC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38745" yWindow="1305" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -85,7 +85,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -389,7 +389,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
-        <v>0.29166666666666669</v>
+        <v>46296.291666666664</v>
       </c>
       <c r="B2">
         <v>1.44</v>
@@ -403,7 +403,8 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>0.30208333333333331</v>
+        <f>A2+1/24/4</f>
+        <v>46296.302083333328</v>
       </c>
       <c r="B3">
         <v>1.5</v>
@@ -417,7 +418,8 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
-        <v>0.3125</v>
+        <f t="shared" ref="A4:A67" si="0">A3+1/24/4</f>
+        <v>46296.312499999993</v>
       </c>
       <c r="B4">
         <v>1.59</v>
@@ -431,7 +433,8 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
-        <v>0.32291666666666669</v>
+        <f t="shared" si="0"/>
+        <v>46296.322916666657</v>
       </c>
       <c r="B5">
         <v>1.47</v>
@@ -445,7 +448,8 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
-        <v>0.33333333333333331</v>
+        <f t="shared" si="0"/>
+        <v>46296.333333333321</v>
       </c>
       <c r="B6">
         <v>1.55</v>
@@ -459,7 +463,8 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
-        <v>0.34375</v>
+        <f t="shared" si="0"/>
+        <v>46296.343749999985</v>
       </c>
       <c r="B7">
         <v>1.36</v>
@@ -473,7 +478,8 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
-        <v>0.35416666666666669</v>
+        <f t="shared" si="0"/>
+        <v>46296.35416666665</v>
       </c>
       <c r="B8">
         <v>1.42</v>
@@ -487,7 +493,8 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
-        <v>0.36458333333333331</v>
+        <f t="shared" si="0"/>
+        <v>46296.364583333314</v>
       </c>
       <c r="B9">
         <v>1.48</v>
@@ -501,7 +508,8 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
-        <v>0.375</v>
+        <f t="shared" si="0"/>
+        <v>46296.374999999978</v>
       </c>
       <c r="B10">
         <v>1.42</v>
@@ -515,7 +523,8 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
-        <v>0.38541666666666669</v>
+        <f t="shared" si="0"/>
+        <v>46296.385416666642</v>
       </c>
       <c r="B11">
         <v>1.32</v>
@@ -529,7 +538,8 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
-        <v>0.39583333333333331</v>
+        <f t="shared" si="0"/>
+        <v>46296.395833333307</v>
       </c>
       <c r="B12">
         <v>1.56</v>
@@ -543,7 +553,8 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
-        <v>0.40625</v>
+        <f t="shared" si="0"/>
+        <v>46296.406249999971</v>
       </c>
       <c r="B13">
         <v>1.21</v>
@@ -557,7 +568,8 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
-        <v>0.41666666666666669</v>
+        <f t="shared" si="0"/>
+        <v>46296.416666666635</v>
       </c>
       <c r="B14">
         <v>1.45</v>
@@ -571,7 +583,8 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
-        <v>0.42708333333333331</v>
+        <f t="shared" si="0"/>
+        <v>46296.427083333299</v>
       </c>
       <c r="B15">
         <v>2</v>
@@ -585,7 +598,8 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
-        <v>0.4375</v>
+        <f t="shared" si="0"/>
+        <v>46296.437499999964</v>
       </c>
       <c r="B16">
         <v>2.06</v>
@@ -599,7 +613,8 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
-        <v>0.44791666666666669</v>
+        <f t="shared" si="0"/>
+        <v>46296.447916666628</v>
       </c>
       <c r="B17">
         <v>1.41</v>
@@ -613,7 +628,8 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
-        <v>0.45833333333333331</v>
+        <f t="shared" si="0"/>
+        <v>46296.458333333292</v>
       </c>
       <c r="B18">
         <v>1.42</v>
@@ -627,7 +643,8 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
-        <v>0.46875</v>
+        <f t="shared" si="0"/>
+        <v>46296.468749999956</v>
       </c>
       <c r="B19">
         <v>1.24</v>
@@ -641,7 +658,8 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
-        <v>0.47916666666666669</v>
+        <f t="shared" si="0"/>
+        <v>46296.479166666621</v>
       </c>
       <c r="B20">
         <v>1.5</v>
@@ -655,7 +673,8 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
-        <v>0.48958333333333331</v>
+        <f t="shared" si="0"/>
+        <v>46296.489583333285</v>
       </c>
       <c r="B21">
         <v>1.36</v>
@@ -669,7 +688,8 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
-        <v>0.5</v>
+        <f t="shared" si="0"/>
+        <v>46296.499999999949</v>
       </c>
       <c r="B22">
         <v>1.55</v>
@@ -683,7 +703,8 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
-        <v>0.51041666666666663</v>
+        <f t="shared" si="0"/>
+        <v>46296.510416666613</v>
       </c>
       <c r="B23">
         <v>1.58</v>
@@ -697,7 +718,8 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
-        <v>0.52083333333333337</v>
+        <f t="shared" si="0"/>
+        <v>46296.520833333278</v>
       </c>
       <c r="B24">
         <v>2</v>
@@ -711,7 +733,8 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
-        <v>0.53125</v>
+        <f t="shared" si="0"/>
+        <v>46296.531249999942</v>
       </c>
       <c r="B25">
         <v>1.41</v>
@@ -725,7 +748,8 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
-        <v>0.54166666666666663</v>
+        <f t="shared" si="0"/>
+        <v>46296.541666666606</v>
       </c>
       <c r="B26">
         <v>1.46</v>
@@ -739,7 +763,8 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
-        <v>0.55208333333333337</v>
+        <f t="shared" si="0"/>
+        <v>46296.55208333327</v>
       </c>
       <c r="B27">
         <v>1.51</v>
@@ -753,7 +778,8 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>0.5625</v>
+        <f t="shared" si="0"/>
+        <v>46296.562499999935</v>
       </c>
       <c r="B28">
         <v>1.42</v>
@@ -767,7 +793,8 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>0.57291666666666663</v>
+        <f t="shared" si="0"/>
+        <v>46296.572916666599</v>
       </c>
       <c r="B29">
         <v>1.37</v>
@@ -781,7 +808,8 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>0.58333333333333337</v>
+        <f t="shared" si="0"/>
+        <v>46296.583333333263</v>
       </c>
       <c r="B30">
         <v>6</v>
@@ -795,7 +823,8 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
-        <v>0.59375</v>
+        <f t="shared" si="0"/>
+        <v>46296.593749999927</v>
       </c>
       <c r="B31">
         <v>6.16</v>
@@ -809,7 +838,8 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <v>0.60416666666666663</v>
+        <f t="shared" si="0"/>
+        <v>46296.604166666591</v>
       </c>
       <c r="B32">
         <v>5.12</v>
@@ -823,7 +853,8 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>0.61458333333333337</v>
+        <f t="shared" si="0"/>
+        <v>46296.614583333256</v>
       </c>
       <c r="B33">
         <v>7.07</v>
@@ -837,7 +868,8 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <v>0.625</v>
+        <f t="shared" si="0"/>
+        <v>46296.62499999992</v>
       </c>
       <c r="B34">
         <v>7</v>
@@ -851,7 +883,8 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
-        <v>0.63541666666666663</v>
+        <f t="shared" si="0"/>
+        <v>46296.635416666584</v>
       </c>
       <c r="B35">
         <v>7.01</v>
@@ -865,7 +898,8 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>0.64583333333333337</v>
+        <f t="shared" si="0"/>
+        <v>46296.645833333248</v>
       </c>
       <c r="B36">
         <v>7.34</v>
@@ -879,7 +913,8 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>0.65625</v>
+        <f t="shared" si="0"/>
+        <v>46296.656249999913</v>
       </c>
       <c r="B37">
         <v>7.45</v>
@@ -893,7 +928,8 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
-        <v>0.66666666666666663</v>
+        <f t="shared" si="0"/>
+        <v>46296.666666666577</v>
       </c>
       <c r="B38">
         <v>9.02</v>
@@ -907,7 +943,8 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
-        <v>0.67708333333333337</v>
+        <f t="shared" si="0"/>
+        <v>46296.677083333241</v>
       </c>
       <c r="B39">
         <v>8.43</v>
@@ -921,7 +958,8 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
-        <v>0.6875</v>
+        <f t="shared" si="0"/>
+        <v>46296.687499999905</v>
       </c>
       <c r="B40">
         <v>9.33</v>
@@ -935,7 +973,8 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
-        <v>0.69791666666666663</v>
+        <f t="shared" si="0"/>
+        <v>46296.69791666657</v>
       </c>
       <c r="B41">
         <v>10.23</v>
@@ -949,7 +988,8 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
-        <v>0.70833333333333337</v>
+        <f t="shared" si="0"/>
+        <v>46296.708333333234</v>
       </c>
       <c r="B42">
         <v>9.42</v>
@@ -963,7 +1003,8 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
-        <v>0.71875</v>
+        <f t="shared" si="0"/>
+        <v>46296.718749999898</v>
       </c>
       <c r="B43">
         <v>9.41</v>
@@ -977,7 +1018,8 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
-        <v>0.72916666666666663</v>
+        <f t="shared" si="0"/>
+        <v>46296.729166666562</v>
       </c>
       <c r="B44">
         <v>9.06</v>
@@ -991,7 +1033,8 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
-        <v>0.73958333333333337</v>
+        <f t="shared" si="0"/>
+        <v>46296.739583333227</v>
       </c>
       <c r="B45">
         <v>10.53</v>
@@ -1005,7 +1048,8 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
-        <v>0.75</v>
+        <f t="shared" si="0"/>
+        <v>46296.749999999891</v>
       </c>
       <c r="B46">
         <v>9.33</v>
@@ -1019,7 +1063,8 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>0.76041666666666663</v>
+        <f t="shared" si="0"/>
+        <v>46296.760416666555</v>
       </c>
       <c r="B47">
         <v>8.2100000000000009</v>
@@ -1033,7 +1078,8 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
-        <v>0.77083333333333337</v>
+        <f t="shared" si="0"/>
+        <v>46296.770833333219</v>
       </c>
       <c r="B48">
         <v>7.33</v>
@@ -1047,7 +1093,8 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
-        <v>0.78125</v>
+        <f t="shared" si="0"/>
+        <v>46296.781249999884</v>
       </c>
       <c r="B49">
         <v>7.28</v>
@@ -1061,7 +1108,8 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>0.79166666666666663</v>
+        <f t="shared" si="0"/>
+        <v>46296.791666666548</v>
       </c>
       <c r="B50">
         <v>5.52</v>
@@ -1075,7 +1123,8 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>0.80208333333333337</v>
+        <f t="shared" si="0"/>
+        <v>46296.802083333212</v>
       </c>
       <c r="B51">
         <v>7.11</v>
@@ -1089,7 +1138,8 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
-        <v>0.8125</v>
+        <f t="shared" si="0"/>
+        <v>46296.812499999876</v>
       </c>
       <c r="B52">
         <v>6.17</v>
@@ -1103,7 +1153,8 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>0.82291666666666663</v>
+        <f t="shared" si="0"/>
+        <v>46296.822916666541</v>
       </c>
       <c r="B53">
         <v>7.12</v>
@@ -1117,7 +1168,8 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
-        <v>0.83333333333333337</v>
+        <f t="shared" si="0"/>
+        <v>46296.833333333205</v>
       </c>
       <c r="B54">
         <v>6.19</v>
@@ -1131,7 +1183,8 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
-        <v>0.84375</v>
+        <f t="shared" si="0"/>
+        <v>46296.843749999869</v>
       </c>
       <c r="B55">
         <v>7.02</v>
@@ -1145,7 +1198,8 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>0.85416666666666663</v>
+        <f t="shared" si="0"/>
+        <v>46296.854166666533</v>
       </c>
       <c r="B56">
         <v>6.4</v>
@@ -1159,7 +1213,8 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
-        <v>0.86458333333333337</v>
+        <f t="shared" si="0"/>
+        <v>46296.864583333198</v>
       </c>
       <c r="B57">
         <v>6.22</v>
@@ -1173,7 +1228,8 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
-        <v>0.875</v>
+        <f t="shared" si="0"/>
+        <v>46296.874999999862</v>
       </c>
       <c r="B58">
         <v>9.06</v>
@@ -1187,7 +1243,8 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
-        <v>0.88541666666666663</v>
+        <f t="shared" si="0"/>
+        <v>46296.885416666526</v>
       </c>
       <c r="B59">
         <v>9.02</v>
@@ -1201,7 +1258,8 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>0.89583333333333337</v>
+        <f t="shared" si="0"/>
+        <v>46296.89583333319</v>
       </c>
       <c r="B60">
         <v>9.3000000000000007</v>
@@ -1215,7 +1273,8 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
-        <v>0.90625</v>
+        <f t="shared" si="0"/>
+        <v>46296.906249999854</v>
       </c>
       <c r="B61">
         <v>9.35</v>
@@ -1229,7 +1288,8 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
-        <v>0.91666666666666663</v>
+        <f t="shared" si="0"/>
+        <v>46296.916666666519</v>
       </c>
       <c r="B62">
         <v>9.49</v>
@@ -1243,7 +1303,8 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
-        <v>0.92708333333333337</v>
+        <f t="shared" si="0"/>
+        <v>46296.927083333183</v>
       </c>
       <c r="B63">
         <v>9.5500000000000007</v>
@@ -1257,7 +1318,8 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
-        <v>0.9375</v>
+        <f t="shared" si="0"/>
+        <v>46296.937499999847</v>
       </c>
       <c r="B64">
         <v>9.11</v>
@@ -1271,7 +1333,8 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <v>0.94791666666666663</v>
+        <f t="shared" si="0"/>
+        <v>46296.947916666511</v>
       </c>
       <c r="B65">
         <v>9.39</v>
@@ -1285,7 +1348,8 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <v>0.95833333333333337</v>
+        <f t="shared" si="0"/>
+        <v>46296.958333333176</v>
       </c>
       <c r="B66">
         <v>8.35</v>
@@ -1299,7 +1363,8 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
-        <v>0.96875</v>
+        <f t="shared" si="0"/>
+        <v>46296.96874999984</v>
       </c>
       <c r="B67">
         <v>8.25</v>
@@ -1313,7 +1378,8 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <v>0.97916666666666663</v>
+        <f t="shared" ref="A68:A97" si="1">A67+1/24/4</f>
+        <v>46296.979166666504</v>
       </c>
       <c r="B68">
         <v>8.1300000000000008</v>
@@ -1327,7 +1393,8 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <v>0.98958333333333337</v>
+        <f t="shared" si="1"/>
+        <v>46296.989583333168</v>
       </c>
       <c r="B69">
         <v>8.2899999999999991</v>
@@ -1341,7 +1408,8 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>46296.999999999833</v>
       </c>
       <c r="B70">
         <v>6.35</v>
@@ -1355,7 +1423,8 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <v>1.0416666666666666E-2</v>
+        <f t="shared" si="1"/>
+        <v>46297.010416666497</v>
       </c>
       <c r="B71">
         <v>5.43</v>
@@ -1369,7 +1438,8 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
-        <v>2.0833333333333332E-2</v>
+        <f t="shared" si="1"/>
+        <v>46297.020833333161</v>
       </c>
       <c r="B72">
         <v>6.28</v>
@@ -1383,7 +1453,8 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
-        <v>3.125E-2</v>
+        <f t="shared" si="1"/>
+        <v>46297.031249999825</v>
       </c>
       <c r="B73">
         <v>6.44</v>
@@ -1397,7 +1468,8 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
-        <v>4.1666666666666664E-2</v>
+        <f t="shared" si="1"/>
+        <v>46297.04166666649</v>
       </c>
       <c r="B74">
         <v>6.05</v>
@@ -1411,7 +1483,8 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
-        <v>5.2083333333333336E-2</v>
+        <f t="shared" si="1"/>
+        <v>46297.052083333154</v>
       </c>
       <c r="B75">
         <v>1.55</v>
@@ -1425,7 +1498,8 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
-        <v>6.25E-2</v>
+        <f t="shared" si="1"/>
+        <v>46297.062499999818</v>
       </c>
       <c r="B76">
         <v>1.39</v>
@@ -1439,7 +1513,8 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
-        <v>7.2916666666666671E-2</v>
+        <f t="shared" si="1"/>
+        <v>46297.072916666482</v>
       </c>
       <c r="B77">
         <v>1.3</v>
@@ -1453,7 +1528,8 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
-        <v>8.3333333333333329E-2</v>
+        <f t="shared" si="1"/>
+        <v>46297.083333333147</v>
       </c>
       <c r="B78">
         <v>1.45</v>
@@ -1467,7 +1543,8 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
-        <v>9.375E-2</v>
+        <f t="shared" si="1"/>
+        <v>46297.093749999811</v>
       </c>
       <c r="B79">
         <v>1.52</v>
@@ -1481,7 +1558,8 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
-        <v>0.10416666666666667</v>
+        <f t="shared" si="1"/>
+        <v>46297.104166666475</v>
       </c>
       <c r="B80">
         <v>2.0499999999999998</v>
@@ -1495,7 +1573,8 @@
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
-        <v>0.11458333333333333</v>
+        <f t="shared" si="1"/>
+        <v>46297.114583333139</v>
       </c>
       <c r="B81">
         <v>1.39</v>
@@ -1509,7 +1588,8 @@
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
-        <v>0.125</v>
+        <f t="shared" si="1"/>
+        <v>46297.124999999804</v>
       </c>
       <c r="B82">
         <v>2.0499999999999998</v>
@@ -1523,7 +1603,8 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
-        <v>0.13541666666666666</v>
+        <f t="shared" si="1"/>
+        <v>46297.135416666468</v>
       </c>
       <c r="B83">
         <v>1.52</v>
@@ -1537,7 +1618,8 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
-        <v>0.14583333333333334</v>
+        <f t="shared" si="1"/>
+        <v>46297.145833333132</v>
       </c>
       <c r="B84">
         <v>1.45</v>
@@ -1551,7 +1633,8 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
-        <v>0.15625</v>
+        <f t="shared" si="1"/>
+        <v>46297.156249999796</v>
       </c>
       <c r="B85">
         <v>1.42</v>
@@ -1565,7 +1648,8 @@
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="1">
-        <v>0.16666666666666666</v>
+        <f t="shared" si="1"/>
+        <v>46297.166666666461</v>
       </c>
       <c r="B86">
         <v>1.52</v>
@@ -1579,7 +1663,8 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
-        <v>0.17708333333333334</v>
+        <f t="shared" si="1"/>
+        <v>46297.177083333125</v>
       </c>
       <c r="B87">
         <v>2.08</v>
@@ -1593,7 +1678,8 @@
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
-        <v>0.1875</v>
+        <f t="shared" si="1"/>
+        <v>46297.187499999789</v>
       </c>
       <c r="B88">
         <v>1.33</v>
@@ -1607,7 +1693,8 @@
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
-        <v>0.19791666666666666</v>
+        <f t="shared" si="1"/>
+        <v>46297.197916666453</v>
       </c>
       <c r="B89">
         <v>1.47</v>
@@ -1621,7 +1708,8 @@
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="1">
-        <v>0.20833333333333334</v>
+        <f t="shared" si="1"/>
+        <v>46297.208333333117</v>
       </c>
       <c r="B90">
         <v>1.49</v>
@@ -1635,7 +1723,8 @@
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
-        <v>0.21875</v>
+        <f t="shared" si="1"/>
+        <v>46297.218749999782</v>
       </c>
       <c r="B91">
         <v>1.47</v>
@@ -1649,7 +1738,8 @@
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="1">
-        <v>0.22916666666666666</v>
+        <f t="shared" si="1"/>
+        <v>46297.229166666446</v>
       </c>
       <c r="B92">
         <v>1.51</v>
@@ -1663,7 +1753,8 @@
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="1">
-        <v>0.23958333333333334</v>
+        <f t="shared" si="1"/>
+        <v>46297.23958333311</v>
       </c>
       <c r="B93">
         <v>1.51</v>
@@ -1677,7 +1768,8 @@
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
-        <v>0.25</v>
+        <f t="shared" si="1"/>
+        <v>46297.249999999774</v>
       </c>
       <c r="B94">
         <v>1.45</v>
@@ -1691,7 +1783,8 @@
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="1">
-        <v>0.26041666666666669</v>
+        <f t="shared" si="1"/>
+        <v>46297.260416666439</v>
       </c>
       <c r="B95">
         <v>1.58</v>
@@ -1705,7 +1798,8 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
-        <v>0.27083333333333331</v>
+        <f t="shared" si="1"/>
+        <v>46297.270833333103</v>
       </c>
       <c r="B96">
         <v>1.42</v>
@@ -1719,7 +1813,8 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
-        <v>0.28125</v>
+        <f t="shared" si="1"/>
+        <v>46297.281249999767</v>
       </c>
       <c r="B97">
         <v>1.56</v>

</xml_diff>